<commit_message>
docs(security): correct G-10 public operations, G-15 PKCE/logout findings; widen register sync check
- G-10 / IA-2 / AC-3: GET /op/configuration and GET /op/definition declare
  security: [] and answer unauthenticated; AC-3 downgraded to Partially.
- G-15: PKCE S256 is always used (STIGMAN_CLIENT_STRICT_PKCE only gates the
  metadata check); the real gap is that the worker logout handler does not
  clear shared-worker tokens, so a second tab keeps the access token until exp.
  Moved to Phase 1. Auth sequence diagram and test plan updated to match.
- --check now compares crosswalk status and gap refs, pillar gap lists and
  roadmap phase gap lists against the data, not only IDs and counts.

Co-Authored-By: Erik Rozi <erik.rozi@cognition.ai>
</commit_message>
<xml_diff>
--- a/docs/security/icam-zero-trust/ICAM-ZT-Gap-Register.xlsx
+++ b/docs/security/icam-zero-trust/ICAM-ZT-Gap-Register.xlsx
@@ -1115,7 +1115,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Scope matching — api/source/utils/auth.js:161-185 (validateOauthSecurity); api/source/specification/stig-manager.yaml:10892-10900 (securitySchemes)</t>
+          <t>Scope matching — api/source/utils/auth.js:161-185 (validateOauthSecurity); api/source/specification/stig-manager.yaml:10892-10900 (securitySchemes), :3753 and :3767 (security: [] on /op/configuration and /op/definition)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1130,22 +1130,22 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Every operation in the OpenAPI specification declares required `stig-manager:*` scopes and the handler is enforced by express-openapi-validator (middlewares.js:111). Granted scopes match if equal or if the granted scope is a prefix of the required scope by colon-separated tokens (auth.js:170-178), so `stig-manager:collection` satisfies `stig-manager:collection:read`.</t>
+          <t>Every operation in the OpenAPI specification declares required `stig-manager:*` scopes except two that declare `security: []`: GET /op/configuration and GET /op/definition (stig-manager.yaml:3753, 3767). validateToken only verifies a token when one is present (auth.js:86-87), so those two operations answer unauthenticated requests; /op/configuration returns the API version, commit, last migration and every row of the `config` table (controllers/Operation.js:8-13; OperationService.js:19-27), and /op/definition returns the OpenAPI document. All other operations are enforced by express-openapi-validator (middlewares.js:111). Granted scopes match if equal or if the granted scope is a prefix of the required scope by colon-separated tokens (auth.js:170-178), so `stig-manager:collection` satisfies `stig-manager:collection:read`.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Scope enforcement is well-structured, but the prefix rule means a broad parent scope grants every child operation; there is no documentation of the minimum scope set per role and no test asserting that unexpected scope strings are rejected.</t>
+          <t>Two operations are intentionally unauthenticated and are not identified as public exceptions in the security documentation; the `config` table contents are disclosed to anyone who can reach the API. For authenticated operations the prefix rule means a broad parent scope grants every child operation; there is no documentation of the minimum scope set per role and no test asserting that unexpected scope strings are rejected.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>L — Behaviour is deliberate and consistent; the residual risk is over-broad scope issuance at the IdP.</t>
+          <t>L — The public operations disclose version and configuration values but no user or assessment data, and the client needs /op/configuration before login; the authenticated path is deliberate and consistent. Residual risk is over-broad scope issuance at the IdP and disclosure of any sensitive value a deployment places in `config`.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Publish a least-privilege scope matrix (role → minimum scopes) in authentication.rst; add unit tests for prefix matching and rejection of unrelated scopes; recommend IdP client scope restrictions per client.</t>
+          <t>Document /op/configuration and /op/definition as the only public operations and add a test that fails if any other operation declares `security: []`; restrict /op/configuration to the keys the client needs before login; publish a least-privilege scope matrix (role → minimum scopes) in authentication.rst; add unit tests for prefix matching and rejection of unrelated scopes; recommend IdP client scope restrictions per client.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Web client authorization flow — client/src/js/workers/oidc-worker.js:205 (strict PKCE check), :267 (S256), :420-421 (audience and claim validation), :115-118 (logout via end_session_endpoint); api/source/utils/config.js:45 (STIGMAN_CLIENT_STRICT_PKCE)</t>
+          <t>Web client authorization flow — client/src/js/workers/oidc-worker.js:205 (strict PKCE metadata check), :266-267 (S256 challenge), :63 (code_verifier), :114-119 (logout returns end_session_endpoint only), :519-525 (clearTokens); client/src/js/init.js:217-223 (page logout wrapper); api/source/utils/config.js:45 (STIGMAN_CLIENT_STRICT_PKCE)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1440,27 +1440,27 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Authorization Code with PKCE S256 is enforced when strictPkce is true (default) and the worker refuses providers that do not advertise S256 (oidc-worker.js:205, 267). Tokens are held in worker memory, not in storage. Logout redirects to the provider end_session_endpoint (oidc-worker.js:115-118). PKCE can be disabled by setting STIGMAN_CLIENT_STRICT_PKCE=false (config.js:45).</t>
+          <t>Authorization Code with PKCE S256 is always used: every authorization request carries code_challenge_method=S256 (oidc-worker.js:266-267) and every code exchange carries code_verifier (oidc-worker.js:63). STIGMAN_CLIENT_STRICT_PKCE=false (config.js:45) only skips the check that provider metadata advertises S256 (oidc-worker.js:205); it does not disable PKCE. Tokens are held in shared-worker memory, not in storage. The worker logout handler returns the provider end_session_endpoint and does not call clearTokens (oidc-worker.js:114-119); the page wrapper nulls its own token fields and redirects (init.js:217-223). clearTokens with broadcast exists and is used on refresh failure (oidc-worker.js:329, 569, 583).</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>The flow is current-practice; the only gap is that strict PKCE is a runtime switch rather than fixed, and logout does not revoke the refresh token at the IdP (relies on end-session).</t>
+          <t>Logout does not clear the access and refresh tokens held by the shared worker and does not revoke the refresh token at the IdP. While another tab keeps the shared worker alive, that tab can continue to obtain the unchanged access token after a logout in a sibling tab; local termination relies on token expiry and on the IdP end-session redirect.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>L — Defaults are secure; risk arises only if a deployment disables strict PKCE.</t>
+          <t>L — Requires an already-authenticated browser with a second open tab; the access token still expires at `exp` and the IdP session is ended by the redirect. Contained to the client.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Remove or deprecate the option to disable strict PKCE in production builds; call the IdP revocation endpoint (if advertised) for the refresh token on logout; document the required IdP client settings (public client, PKCE required, no implicit flow).</t>
+          <t>In the worker logout handler call clearTokens(true) before returning the redirect and test the multi-tab case; call the IdP revocation endpoint (if advertised) for the refresh token on logout; document the required IdP client settings (public client, PKCE required, no implicit flow).</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>ISSM</t>
+          <t>ISSM; Program Office (client change)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 1</t>
         </is>
       </c>
     </row>
@@ -2239,12 +2239,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>All API access requires a bearer token validated against the IdP JWKS (auth.js:84-100). Identification is by username claim, not persistent identifier (auth.js:110-111).</t>
+          <t>All API operations require a bearer token validated against the IdP JWKS (auth.js:84-100) except GET /op/configuration and GET /op/definition, which declare security: [] (stig-manager.yaml:3753, 3767). Identification is by username claim, not persistent identifier (auth.js:110-111).</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>G-05, G-17</t>
+          <t>G-05, G-10, G-17</t>
         </is>
       </c>
     </row>
@@ -2477,12 +2477,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Satisfied</t>
+          <t>Partially</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>OpenAPI scope enforcement on every operation (middlewares.js:111, auth.js:161-185) and collection-grant checks (Collection.js:389-405).</t>
+          <t>OpenAPI scope enforcement on every operation (middlewares.js:111, auth.js:161-185) and collection-grant checks (Collection.js:389-405), with two documented-in-spec public exceptions: /op/configuration and /op/definition (stig-manager.yaml:3753, 3767) return version, `config` table rows and the API definition without authentication.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Logout via IdP end_session_endpoint (oidc-worker.js:115-118); no server-side revocation; token valid until exp.</t>
+          <t>Logout returns the IdP end_session_endpoint without clearing worker-held tokens (oidc-worker.js:114-119); no refresh-token revocation; access token valid until exp.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>G-01, G-02, G-09, G-10, G-11, G-12, G-14, G-16, G-20, G-24</t>
+          <t>G-01, G-02, G-09, G-10, G-11, G-12, G-14, G-15, G-16, G-20, G-24</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>G-03, G-04, G-05, G-06, G-07, G-08, G-13, G-15, G-17, G-21, G-22, G-23</t>
+          <t>G-03, G-04, G-05, G-06, G-07, G-08, G-13, G-17, G-21, G-22, G-23</t>
         </is>
       </c>
     </row>

</xml_diff>